<commit_message>
Simplify OCR upload workflow
</commit_message>
<xml_diff>
--- a/samples/expected_orders.xlsx
+++ b/samples/expected_orders.xlsx
@@ -413,71 +413,41 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I2"/>
+  <dimension ref="A1:D2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="20" customWidth="1" min="1" max="1"/>
-    <col width="19" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
-    <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="21" customWidth="1" min="7" max="7"/>
-    <col width="18" customWidth="1" min="8" max="8"/>
-    <col width="60" customWidth="1" min="9" max="9"/>
+    <col width="8" customWidth="1" min="1" max="1"/>
+    <col width="58" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>订单编号</t>
+          <t>序号</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>商品名称</t>
+          <t>商品信息</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>商品规格</t>
+          <t>实付款</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>数量</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>订单金额</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>订单状态</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>下单时间</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr">
-        <is>
           <t>截图文件</t>
-        </is>
-      </c>
-      <c r="I1" t="inlineStr">
-        <is>
-          <t>OCR全文</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>123456789012345678</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -487,46 +457,12 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>黑色 XL</t>
+          <t>39.90</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>39.90</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>待收货</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>2026-07-08 20:15:30</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
           <t>sample_order.png</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>拼多多订单详情
-待收货
-南极人男士短袖T恤夏季纯棉宽松上衣
-黑色 XL x1
-7天无理由退货极速退款
-实付款￥39.90
-2026-07-08 20:15:30
-123456789012345678
-查看物流联系卖家
-申请售后</t>
         </is>
       </c>
     </row>

</xml_diff>